<commit_message>
Fix squad assignments: Chella to CSK, Avengers captain
- Madhusudan Chella (5CF2) moves from DIGI TITANS to Colruyt Super Kings in
  data/auction_log_2026.csv; Nagaraju Muddana's price goes back to 280 (the
  earlier trim to 275 was only needed while Chella inflated the Digititans
  column). Digititans 970, CSK 1000.
- Regenerate data/CPL_2026_PreAuction_Template.xlsx and 2026_pre_auction_insert.sql
  from the current CPL2026.xlsx, which corrects the stale Avengers captain: Siva
  Naga Kishore Raju Samanthapudi (5DXX) is Captain, Pradeep Kumar Pala is Squad.
- squads2026.js and the apply/verify SQL regenerated to match.

Every one of the 68 placed players verified against the owner's team log.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CPL_2026_PreAuction_Template.xlsx
+++ b/data/CPL_2026_PreAuction_Template.xlsx
@@ -544,10 +544,10 @@
         <v>Avengers</v>
       </c>
       <c r="B2" t="str">
-        <v>2BJB</v>
+        <v>5DXX</v>
       </c>
       <c r="C2" t="str">
-        <v>Pradeep Kumar Pala</v>
+        <v>Siva Naga Kishore Raju Samanthapudi</v>
       </c>
       <c r="D2" t="str">
         <v>All-rounder</v>
@@ -562,7 +562,7 @@
         <v>Unknown</v>
       </c>
       <c r="H2" t="str">
-        <v>2BJB.jpg</v>
+        <v>5DXX.jpg</v>
       </c>
       <c r="I2" t="str">
         <v>All-rounder</v>
@@ -631,10 +631,10 @@
         <v>Avengers</v>
       </c>
       <c r="B5" t="str">
-        <v>5DXX</v>
+        <v>2BJB</v>
       </c>
       <c r="C5" t="str">
-        <v>Siva Naga Kishore Raju Samanthapudi</v>
+        <v>Pradeep Kumar Pala</v>
       </c>
       <c r="D5" t="str">
         <v>All-rounder</v>
@@ -649,7 +649,7 @@
         <v>Unknown</v>
       </c>
       <c r="H5" t="str">
-        <v>5DXX.jpg</v>
+        <v>2BJB.jpg</v>
       </c>
       <c r="I5" t="str">
         <v>All-rounder</v>

</xml_diff>